<commit_message>
docs: refresh M1 self-assessment after resend, ABHA address and success-screen fixes
Five mandatory rows move from FAIL to NOT TESTED (resend rule x3, ABHA address policy,
ABHA number on the creation screen). Remaining mandatory FAILs: ABHA-address login via
Aadhaar/mobile OTP and Scan & Share.
</commit_message>
<xml_diff>
--- a/docs/M1_ABHA_Assessment_Self-Check.xlsx
+++ b/docs/M1_ABHA_Assessment_Self-Check.xlsx
@@ -2564,12 +2564,12 @@
       <c r="J27" s="148" t="n"/>
       <c r="K27" s="185" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="L27" s="186" t="inlineStr">
         <is>
-          <t>Resend exists but is allowed after 30 s with no limit. The sheet wants at most 2 resends, each after 60 s. Small change.</t>
+          <t>Resend now becomes available after 60 s and is limited to 2 per OTP request (button shows how many are left, then 'Resend limit reached'). Built, not yet tried in the browser.</t>
         </is>
       </c>
       <c r="M27" s="15" t="n"/>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="L30" s="186" t="inlineStr">
         <is>
-          <t>After creation, an OTP is sent to the communication mobile (enrol request/otp + auth/byAbdm), with resend. Built, but not yet tested with a real OTP.</t>
+          <t>After creation, an OTP is sent to the communication mobile (enrol request/otp + auth/byAbdm); resend follows the 60 s / 2x rule. Built, but not yet tested with a real OTP.</t>
         </is>
       </c>
       <c r="M30" s="8" t="n"/>
@@ -2846,12 +2846,12 @@
       <c r="J31" s="14" t="n"/>
       <c r="K31" s="185" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="L31" s="186" t="inlineStr">
         <is>
-          <t>Suggestions and a custom address are built, but our rule is 4-18 characters (sheet: min 8, max 18) and the rules show only after an error, not beside the field. Not tested live.</t>
+          <t>Suggestions and a custom address are built. Rules now follow the sheet (8-18 characters, one dot and/or underscore, not at the ends) and are printed beside the field; the server enforces the same. Not yet tested live.</t>
         </is>
       </c>
       <c r="M31" s="12" t="n"/>
@@ -2911,12 +2911,12 @@
       <c r="J32" s="148" t="n"/>
       <c r="K32" s="185" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="L32" s="186" t="inlineStr">
         <is>
-          <t>The number and address show on the patient record, but not on the creation success screen. Show them right after creation.</t>
+          <t>The ABHA number and address now show on the creation screen and again on the success screen. Built, not yet tried in the browser.</t>
         </is>
       </c>
       <c r="M32" s="8" t="n"/>
@@ -5303,7 +5303,7 @@
       </c>
       <c r="L69" s="186" t="inlineStr">
         <is>
-          <t>Link by ABHA number with the OTP sent to the Aadhaar-linked mobile; the profile is fetched and linked after the name/date-of-birth check. Built, not yet tested live. Resend does not follow the 60 s / 2x rule.</t>
+          <t>Link by ABHA number with the OTP sent to the Aadhaar-linked mobile; the profile is fetched and linked after the name/date-of-birth check. Built, not yet tested live. Resend follows the 60 s / 2x rule.</t>
         </is>
       </c>
       <c r="M69" s="8" t="n"/>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="L72" s="186" t="inlineStr">
         <is>
-          <t>Link by ABHA number with the OTP sent to the ABHA's own mobile. Built, not yet tested live. Resend does not follow the 60 s / 2x rule.</t>
+          <t>Link by ABHA number with the OTP sent to the ABHA's own mobile. Built, not yet tested live. Resend follows the 60 s / 2x rule.</t>
         </is>
       </c>
       <c r="M72" s="8" t="n"/>
@@ -5986,12 +5986,12 @@
       <c r="J79" s="148" t="n"/>
       <c r="K79" s="185" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="L79" s="186" t="inlineStr">
         <is>
-          <t>Resend is allowed after 30 s with no limit; the sheet wants max 2 resends, each after 60 s.</t>
+          <t>Resend is available after 60 s, at most 2 per OTP request. Built, not yet tried in the browser.</t>
         </is>
       </c>
       <c r="M79" s="15" t="n"/>
@@ -6358,12 +6358,12 @@
       <c r="J85" s="148" t="n"/>
       <c r="K85" s="185" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="L85" s="186" t="inlineStr">
         <is>
-          <t>Resend is allowed after 30 s with no limit; the sheet wants max 2 resends, each after 60 s.</t>
+          <t>Resend is available after 60 s, at most 2 per OTP request. Built, not yet tried in the browser.</t>
         </is>
       </c>
       <c r="M85" s="15" t="n"/>
@@ -33312,11 +33312,11 @@
     <mergeCell ref="B132:B134"/>
     <mergeCell ref="L132:L134"/>
     <mergeCell ref="L125:L126"/>
+    <mergeCell ref="Q36:Q45"/>
     <mergeCell ref="N125:N126"/>
     <mergeCell ref="O105:O106"/>
-    <mergeCell ref="Q36:Q45"/>
+    <mergeCell ref="N132:N134"/>
     <mergeCell ref="G105:G106"/>
-    <mergeCell ref="N132:N134"/>
     <mergeCell ref="K136:K138"/>
     <mergeCell ref="I105:I106"/>
     <mergeCell ref="H136:H138"/>

</xml_diff>